<commit_message>
rerunning scripts with updated ALFAM2 data submission + adding new.ID to slurry and soil tables
</commit_message>
<xml_diff>
--- a/output/slurry_prop_summary_table.xlsx
+++ b/output/slurry_prop_summary_table.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -367,47 +367,52 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>new.ID</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>pH</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>DM</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>VS</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>TN</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>TAN</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>g kg-1</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>g kg-1</t>
         </is>
@@ -426,25 +431,30 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Trial 1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>7.51 ± 0.04</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>6.2 ± 0.09</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>76.89 ± 0.45</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>2.72 ± 0.02</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>1.13 ± 0.03</t>
         </is>
@@ -463,25 +473,30 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>Trial 1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>8.02 ± 0.02</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>22.49 ± 0.12</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>88.01 ± 0.16</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>3.56 ± 0.3</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>0.43 ± 0.13</t>
         </is>
@@ -500,25 +515,30 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>Trial 1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>7.53 ± 0</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>4.16 ± 0.02</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>70.16 ± 0.31</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>2.48 ± 0</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>1.13 ± 0.09</t>
         </is>
@@ -537,25 +557,30 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>Trial 3</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>7.66 ± 0</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>6.05 ± 0.05</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>76.99 ± 0.41</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>2.72 ± 0.01</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>1.22 ± 0.02</t>
         </is>
@@ -574,25 +599,30 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>Trial 3</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>8.02 ± 0.02</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>21.98 ± 0.41</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>88.58 ± NA</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>3.9 ± 0.4</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>0.43 ± 0.13</t>
         </is>
@@ -611,25 +641,30 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>Trial 3</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t>7.77 ± 0</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>4.22 ± 0.15</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>70.62 ± 0.97</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>2.11 ± 0.26</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>1.31 ± 0.05</t>
         </is>
@@ -648,25 +683,30 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
+          <t>Trial 5</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
           <t>7.92 ± 0.01</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>6.37 ± 0.24</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>77.21 ± 3.1</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>3.1 ± 0.08</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>1.52 ± 0.02</t>
         </is>
@@ -685,25 +725,30 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t>Trial 5</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
           <t>6.6 ± 0.05</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>52.76 ± 0.07</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>88.41 ± 0.04</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>13.28 ± 0.48</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>1.33 ± 0.32</t>
         </is>
@@ -722,25 +767,30 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
+          <t>Trial 5</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
           <t>7.96 ± 0</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>5.35 ± 0.01</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>69.53 ± 0.13</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>2.61 ± 0.06</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>1.06 ± 0.01</t>
         </is>
@@ -759,25 +809,30 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
+          <t>Trial 2</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
           <t>7.16 ± 0</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>3.63 ± 0.07</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>77.25 ± 0.39</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>2.03 ± 0.04</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>1.16 ± 0.03</t>
         </is>
@@ -796,25 +851,30 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
+          <t>Trial 2</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
           <t>8.31 ± 0.04</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>22.3 ± 0.58</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>92.8 ± 0.26</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>2.73 ± 0.06</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>0.71 ± 0.03</t>
         </is>
@@ -833,25 +893,30 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
+          <t>Trial 2</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
           <t>7.36 ± 0</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>2.38 ± 0.01</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>69.77 ± 0.03</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>1.9 ± 0.44</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>1.01 ± 0.05</t>
         </is>
@@ -870,25 +935,30 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
+          <t>Trial 4</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
           <t>7.86 ± 0</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>3.66 ± 0.02</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>68.84 ± 0.41</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>2.07 ± 0.36</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>1.14 ± 0.01</t>
         </is>
@@ -907,25 +977,30 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
+          <t>Trial 4</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
           <t>8.18 ± 0.01</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>21.84 ± 0.27</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>92.58 ± 0.73</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>2.89 ± 0.16</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>1.28 ± 0.09</t>
         </is>
@@ -944,25 +1019,30 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
+          <t>Trial 4</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
           <t>7.66 ± 0.01</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>2.36 ± 0.02</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>77.13 ± 0.26</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>2.13 ± 0</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>1.12 ± 0.11</t>
         </is>
@@ -981,25 +1061,30 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
+          <t>Trial 6</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
           <t>7.08 ± 0.01</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>6.24 ± 0.15</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>79.24 ± 0.51</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>2.02 ± 0.19</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>0.87 ± 0.13</t>
         </is>
@@ -1018,25 +1103,30 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
+          <t>Trial 6</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
           <t>8.84 ± 0.01</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>28.92 ± 0.22</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>92.04 ± 0.14</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>5.81 ± 0.23</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>3.46 ± 0.21</t>
         </is>
@@ -1055,25 +1145,30 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
+          <t>Trial 6</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
           <t>7.88 ± 0.01</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>2.06 ± 0.01</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>59.81 ± 0.27</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>1.51 ± 0.1</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>0.59 ± 0.1</t>
         </is>
@@ -1092,25 +1187,30 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
+          <t>Trial 7</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
           <t>6.88 ± 0</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>45.37 ± 1.62</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>88.21 ± 0.05</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>9.2 ± 0.98</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>1.57 ± 0.17</t>
         </is>
@@ -1129,25 +1229,30 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
+          <t>Trial 7</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
           <t>8.21 ± 0.02</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>45.37 ± 1.62</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>88.21 ± 0.05</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>9.2 ± 0.98</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>1.42</t>
         </is>
@@ -1166,25 +1271,30 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
+          <t>Trial 8</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
           <t>8.08 ± 0</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>5.35 ± 0.01</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>69.53 ± 0.13</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>2.61 ± 0.06</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>1.06 ± 0.01</t>
         </is>
@@ -1203,25 +1313,30 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
+          <t>Trial 8</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
           <t>8.5 ± 0.01</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>5.35 ± 0.01</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>69.53 ± 0.13</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>2.61 ± 0.06</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>1.04</t>
         </is>
@@ -1240,25 +1355,30 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
+          <t>Trial 8</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
           <t>9.2 ± 0.02</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>5.35 ± 0.01</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>69.53 ± 0.13</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>2.61 ± 0.06</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>0.97</t>
         </is>
@@ -1277,25 +1397,30 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
+          <t>Trial 9</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
           <t>7.58 ± 0.01</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>2.06 ± 0.01</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>59.81 ± 0.27</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>1.51 ± 0.1</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>0.59 ± 0.1</t>
         </is>
@@ -1314,25 +1439,30 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
+          <t>Trial 9</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
           <t>7.62 ± 0</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>2.06 ± 0.01</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>59.81 ± 0.27</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>1.51 ± 0.1</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="H27" t="inlineStr">
         <is>
           <t>0.58</t>
         </is>
@@ -1351,25 +1481,30 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
+          <t>Trial 9</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
           <t>8.19 ± 0</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>2.06 ± 0.01</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>59.81 ± 0.27</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>1.51 ± 0.1</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>0.54</t>
         </is>

</xml_diff>